<commit_message>
fix snowflask login and update requirement
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\Spider2-V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B38581-BF9F-4F85-A75D-540791A2434A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3225E94E-3A14-433C-BF58-63C32D8356F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="16800" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="16800" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,10 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>Spider2-V/small (45)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>method</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -46,7 +42,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>coact_15_10_10_20_rag</t>
+    <t>coact_15_15_15_30_rag</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spider2-V/small (44)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -380,33 +380,39 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
         <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>8.8800000000000008</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>27.27</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>31.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add cost and tokens
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\Spider2-V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3225E94E-3A14-433C-BF58-63C32D8356F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B41BD9-0C18-44F0-AC7C-E8899636E62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="16800" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="16800" windowHeight="9670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>method</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -35,9 +35,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>pyautogui_som_gpt-4o-2024-05-13_rag_ef</t>
-  </si>
-  <si>
     <t>coact_15_10_10_20</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -46,7 +43,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Spider2-V/small (44)</t>
+    <t>my_agent_o4_mini_15_rag</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spider2-V/small (68)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>my_agent_o4_mini_50_rag_verbose</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>som_gpt_4o_rag_ef_15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>som_gpt_4o_rag_ef_15_verbose</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>coact_15_20_25_50_rag_verbose</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cost</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tokens</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -372,47 +397,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>4.41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>9.09</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B5">
+        <v>17.649999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>27.27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B6">
+        <v>20.59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
-        <v>31.82</v>
+      <c r="B8">
+        <v>10.29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <v>29.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test osworld, add missing metrics
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\Spider2-V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DF1C97-E4AD-4D7E-967F-C24F798937CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE7FFB1-4121-4906-A336-378E0CD08BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>coact_15_10_10_20</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -68,14 +68,6 @@
   </si>
   <si>
     <t>my_agent_o4mini_15_rag</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>36.88?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>10819783?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -132,9 +124,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -419,7 +413,7 @@
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.83203125" customWidth="1"/>
-    <col min="4" max="4" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -457,9 +451,9 @@
         <v>10.29</v>
       </c>
       <c r="C4">
-        <v>119.1</v>
-      </c>
-      <c r="D4">
+        <v>59.76</v>
+      </c>
+      <c r="D4" s="2">
         <v>19293177</v>
       </c>
     </row>
@@ -484,13 +478,15 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>16.170000000000002</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
+        <v>20.58</v>
+      </c>
+      <c r="C7">
+        <f>0.865*68</f>
+        <v>58.82</v>
+      </c>
+      <c r="D7">
+        <f>408221.25*68</f>
+        <v>27759045</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -503,7 +499,7 @@
     </row>
     <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1">
         <v>36.76</v>
@@ -511,7 +507,7 @@
       <c r="C9" s="1">
         <v>22.12</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="3">
         <v>12368403</v>
       </c>
     </row>

</xml_diff>